<commit_message>
insurer master log and loss cap added
</commit_message>
<xml_diff>
--- a/src/assets/data/SeaAreas.xlsx
+++ b/src/assets/data/SeaAreas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Welcme\PycharmProjects\Edward\src\assets\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E4748007-93D1-423D-94F7-5B6B8D5D19D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BE6FE12-D0C9-41AE-9F0A-FD74C9F5172F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F1B16695-AF8B-490C-9C59-ADE246F2AD8D}"/>
   </bookViews>
@@ -83,21 +83,12 @@
     <t>Central Western Atlantic</t>
   </si>
   <si>
-    <t>Azores</t>
-  </si>
-  <si>
-    <t>Canaries</t>
-  </si>
-  <si>
     <t>Gulf Stream</t>
   </si>
   <si>
     <t>Newfoundland</t>
   </si>
   <si>
-    <t>Cape Verde</t>
-  </si>
-  <si>
     <t>St Lawrence Seaway</t>
   </si>
   <si>
@@ -107,9 +98,6 @@
     <t>Gulf of Guinea</t>
   </si>
   <si>
-    <t>Madeira</t>
-  </si>
-  <si>
     <t>East Greenland</t>
   </si>
   <si>
@@ -120,6 +108,18 @@
   </si>
   <si>
     <t>Baltic Sea</t>
+  </si>
+  <si>
+    <t>Azores Islands area</t>
+  </si>
+  <si>
+    <t>Canary Islands area</t>
+  </si>
+  <si>
+    <t>Cape Verde islands area</t>
+  </si>
+  <si>
+    <t>Madeira island area</t>
   </si>
 </sst>
 </file>
@@ -491,223 +491,223 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A469AC93-760C-4900-B063-B6FC6A3DB4E6}">
-  <dimension ref="B1:C27"/>
+  <dimension ref="A1:B27"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
       <c r="B1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2">
         <v>72</v>
       </c>
-      <c r="C2" t="s">
+      <c r="B2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3">
         <v>114</v>
       </c>
-      <c r="C3" t="s">
+      <c r="B3" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B4">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4">
         <v>55</v>
       </c>
-      <c r="C4" t="s">
+      <c r="B4" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B5">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5">
         <v>67</v>
       </c>
-      <c r="C5" t="s">
+      <c r="B5" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B6">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6">
         <v>56</v>
       </c>
-      <c r="C6" t="s">
+      <c r="B6" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B7">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7">
         <v>57</v>
       </c>
-      <c r="C7" t="s">
+      <c r="B7" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B8">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8">
         <v>69</v>
       </c>
-      <c r="C8" t="s">
+      <c r="B8" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B9">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9">
         <v>1</v>
       </c>
-      <c r="C9" t="s">
+      <c r="B9" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="10" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B10">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10">
         <v>7</v>
       </c>
-      <c r="C10" t="s">
+      <c r="B10" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B11">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11">
         <v>9</v>
       </c>
-      <c r="C11" t="s">
+      <c r="B11" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B12">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12">
         <v>10</v>
       </c>
-      <c r="C12" t="s">
+      <c r="B12" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B13">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13">
         <v>5</v>
       </c>
-      <c r="C13" t="s">
+      <c r="B13" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>6</v>
+      </c>
+      <c r="B14" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="14" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B14">
-        <v>6</v>
-      </c>
-      <c r="C14" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="15" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B15">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15">
         <v>24</v>
       </c>
-      <c r="C15" t="s">
+      <c r="B15" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>2</v>
+      </c>
+      <c r="B16" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>10</v>
+      </c>
+      <c r="B17" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="16" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B16">
-        <v>2</v>
-      </c>
-      <c r="C16" t="s">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>36</v>
+      </c>
+      <c r="B18" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="17" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B17">
-        <v>10</v>
-      </c>
-      <c r="C17" t="s">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>3</v>
+      </c>
+      <c r="B19" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>76</v>
+      </c>
+      <c r="B20" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="18" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B18">
-        <v>36</v>
-      </c>
-      <c r="C18" t="s">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>11</v>
+      </c>
+      <c r="B21" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="19" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B19">
-        <v>3</v>
-      </c>
-      <c r="C19" t="s">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>4</v>
+      </c>
+      <c r="B22" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="20" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B20">
-        <v>76</v>
-      </c>
-      <c r="C20" t="s">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>13</v>
+      </c>
+      <c r="B23" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>43</v>
+      </c>
+      <c r="B24" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="21" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B21">
-        <v>11</v>
-      </c>
-      <c r="C21" t="s">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>93</v>
+      </c>
+      <c r="B25" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="22" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B22">
-        <v>4</v>
-      </c>
-      <c r="C22" t="s">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>70</v>
+      </c>
+      <c r="B26" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="23" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B23">
-        <v>13</v>
-      </c>
-      <c r="C23" t="s">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>21</v>
+      </c>
+      <c r="B27" t="s">
         <v>23</v>
-      </c>
-    </row>
-    <row r="24" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B24">
-        <v>43</v>
-      </c>
-      <c r="C24" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="25" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B25">
-        <v>93</v>
-      </c>
-      <c r="C25" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="26" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B26">
-        <v>69</v>
-      </c>
-      <c r="C26" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="27" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B27">
-        <v>21</v>
-      </c>
-      <c r="C27" t="s">
-        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>